<commit_message>
Fix KCN dashboard bugs: COE premium, valuation label, LNST datalabel
template_kcn.py::calc_valuation_kcn() defaulted specific_risk_premium to
0.02, contradicting its own docstring and the agreed spec (KCN COE = Rf +
β×ERP only, no specific-risk add-on since lease cashflows are stable —
unlike CTCK/banks). Zeroed the default and the two call sites, and fixed
the Excel/PDF labels and captions that still said "+ PBĐT" / a stale
hardcoded "ERP = 5.5%" instead of the actual 7% in use.

kcn.html/app_kcn.js: the valuation snapshot card was labeled "P/B 70% +
P/E 30%" and "RNAV floor" even though the underlying blend is the agreed
40% P/E + 40% P/B + 20% RI — relabeled to match. Also fixed the revenue/
NPAT chart's datalabel plugin, which was printing values on the revenue
bars instead of the NPAT line.

Includes KCN Excel/PDF reports regenerated for IDC/SIP/SZC after these
fixes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/IDC/IDC_KCN_Model_2026-07.xlsx
+++ b/Bao cao/IDC/IDC_KCN_Model_2026-07.xlsx
@@ -119,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,11 +143,12 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -546,7 +547,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Ngày lập: 07/07/2026 23:38</t>
+          <t>Ngày lập: 08/07/2026 22:07</t>
         </is>
       </c>
     </row>
@@ -557,7 +558,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>40000</v>
+        <v>40700</v>
       </c>
     </row>
     <row r="7">
@@ -567,7 +568,7 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>40700</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="8">
@@ -598,7 +599,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1.1511</v>
+        <v>1.1506</v>
       </c>
     </row>
     <row r="11">
@@ -618,7 +619,7 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>0.1083105</v>
+        <v>0.108283</v>
       </c>
     </row>
     <row r="13">
@@ -629,7 +630,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Tự tính toán (1623 phiên)</t>
+          <t>Tự tính toán (1624 phiên)</t>
         </is>
       </c>
     </row>
@@ -657,7 +658,7 @@
         </is>
       </c>
       <c r="C17" s="5" t="n">
-        <v>54092</v>
+        <v>56346</v>
       </c>
     </row>
     <row r="18">
@@ -667,7 +668,7 @@
         </is>
       </c>
       <c r="C18" s="5" t="n">
-        <v>68557</v>
+        <v>68585</v>
       </c>
     </row>
     <row r="19">
@@ -677,7 +678,7 @@
         </is>
       </c>
       <c r="C19" s="10" t="n">
-        <v>53378</v>
+        <v>54285</v>
       </c>
     </row>
     <row r="20">
@@ -687,7 +688,7 @@
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>0.3345</v>
+        <v>0.3338</v>
       </c>
     </row>
     <row r="22">
@@ -762,11 +763,11 @@
         </is>
       </c>
       <c r="B3" s="14" t="n">
-        <v>1.1511</v>
+        <v>1.1506</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Tự tính toán (1623 phiên)</t>
+          <t>Tự tính toán (1624 phiên)</t>
         </is>
       </c>
     </row>
@@ -792,7 +793,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>0.1083105</v>
+        <v>0.108283</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
@@ -897,7 +898,7 @@
         </is>
       </c>
       <c r="B12" s="14" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
@@ -952,7 +953,7 @@
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>40000</v>
+        <v>40700</v>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
@@ -1054,13 +1055,13 @@
         <v>8588.15</v>
       </c>
       <c r="G2" s="17" t="n">
-        <v>9189.32</v>
+        <v>317255.63</v>
       </c>
       <c r="H2" s="17" t="n">
-        <v>9832.57</v>
+        <v>380011.88</v>
       </c>
       <c r="I2" s="17" t="n">
-        <v>10520.85</v>
+        <v>455284.64</v>
       </c>
     </row>
     <row r="3">
@@ -1085,13 +1086,13 @@
         <v>-5528.14</v>
       </c>
       <c r="G3" s="15" t="n">
-        <v>-5818.91</v>
+        <v>-200894.18</v>
       </c>
       <c r="H3" s="15" t="n">
-        <v>-6226.23</v>
+        <v>-240633</v>
       </c>
       <c r="I3" s="15" t="n">
-        <v>-6662.06</v>
+        <v>-288297.59</v>
       </c>
     </row>
     <row r="4">
@@ -1116,13 +1117,13 @@
         <v>14116.29</v>
       </c>
       <c r="G4" s="17" t="n">
-        <v>15008.23</v>
+        <v>518149.81</v>
       </c>
       <c r="H4" s="17" t="n">
-        <v>16058.8</v>
+        <v>620644.88</v>
       </c>
       <c r="I4" s="17" t="n">
-        <v>17182.91</v>
+        <v>743582.23</v>
       </c>
     </row>
     <row r="5">
@@ -1178,13 +1179,13 @@
         <v>2354.08</v>
       </c>
       <c r="G6" s="15" t="n">
-        <v>2501.98</v>
+        <v>86379.22</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>2677.11</v>
+        <v>103465.87</v>
       </c>
       <c r="I6" s="15" t="n">
-        <v>2864.51</v>
+        <v>123960.39</v>
       </c>
     </row>
     <row r="7">
@@ -1263,13 +1264,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1280,15 +1284,30 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
+          <t>2023(CN)A</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>2024(CN)A</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>2025(CN)A</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
           <t>2026E</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>2027E</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="G1" s="12" t="inlineStr">
         <is>
           <t>2028E</t>
         </is>
@@ -1301,13 +1320,22 @@
         </is>
       </c>
       <c r="B2" s="19" t="n">
-        <v>0</v>
+        <v>357.1</v>
       </c>
       <c r="C2" s="19" t="n">
-        <v>0</v>
+        <v>3392.48</v>
       </c>
       <c r="D2" s="19" t="n">
-        <v>0</v>
+        <v>3879.27</v>
+      </c>
+      <c r="E2" s="20" t="n">
+        <v>4073.23</v>
+      </c>
+      <c r="F2" s="20" t="n">
+        <v>4276.9</v>
+      </c>
+      <c r="G2" s="20" t="n">
+        <v>4490.74</v>
       </c>
     </row>
     <row r="3">
@@ -1317,13 +1345,22 @@
         </is>
       </c>
       <c r="B3" s="19" t="n">
-        <v>0</v>
+        <v>1724.63</v>
       </c>
       <c r="C3" s="19" t="n">
-        <v>0</v>
+        <v>4114.55</v>
       </c>
       <c r="D3" s="19" t="n">
-        <v>0</v>
+        <v>3578.99</v>
+      </c>
+      <c r="E3" s="20" t="n">
+        <v>4937.46</v>
+      </c>
+      <c r="F3" s="20" t="n">
+        <v>5924.95</v>
+      </c>
+      <c r="G3" s="20" t="n">
+        <v>7109.94</v>
       </c>
     </row>
     <row r="4">
@@ -1341,6 +1378,15 @@
       <c r="D4" s="19" t="n">
         <v>0</v>
       </c>
+      <c r="E4" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1349,13 +1395,22 @@
         </is>
       </c>
       <c r="B5" s="19" t="n">
-        <v>0</v>
+        <v>73.69</v>
       </c>
       <c r="C5" s="19" t="n">
-        <v>0</v>
+        <v>532.63</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0</v>
+        <v>357.08</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>559.26</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>587.22</v>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>616.59</v>
       </c>
     </row>
     <row r="6">
@@ -1365,13 +1420,22 @@
         </is>
       </c>
       <c r="B6" s="19" t="n">
-        <v>0</v>
+        <v>189.45</v>
       </c>
       <c r="C6" s="19" t="n">
-        <v>0</v>
+        <v>463.84</v>
       </c>
       <c r="D6" s="19" t="n">
-        <v>0</v>
+        <v>480.44</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>576.53</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>691.83</v>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>830.2</v>
       </c>
     </row>
     <row r="7">
@@ -1381,13 +1445,22 @@
         </is>
       </c>
       <c r="B7" s="19" t="n">
-        <v>0</v>
+        <v>10.93</v>
       </c>
       <c r="C7" s="19" t="n">
-        <v>0</v>
+        <v>333.29</v>
       </c>
       <c r="D7" s="19" t="n">
-        <v>0</v>
+        <v>329.19</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>399.95</v>
+      </c>
+      <c r="F7" s="20" t="n">
+        <v>479.94</v>
+      </c>
+      <c r="G7" s="20" t="n">
+        <v>575.9299999999999</v>
       </c>
     </row>
     <row r="8">
@@ -1397,31 +1470,52 @@
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>0</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>0</v>
+        <v>255591</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>0</v>
+        <v>238.95</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>306709.2</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>368051.04</v>
+      </c>
+      <c r="G8" s="20" t="n">
+        <v>441661.25</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>TỔNG DOANH THU</t>
         </is>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="22">
         <f>SUM(B2:B8)</f>
         <v/>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="22">
         <f>SUM(C2:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="21">
+      <c r="D9" s="22">
         <f>SUM(D2:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="22">
+        <f>SUM(E2:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="22">
+        <f>SUM(F2:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="22">
+        <f>SUM(G2:G8)</f>
         <v/>
       </c>
     </row>
@@ -1436,13 +1530,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1453,15 +1550,30 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
+          <t>2023(CN)A</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>2024(CN)A</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>2025(CN)A</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
           <t>2026E</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>2027E</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="G1" s="12" t="inlineStr">
         <is>
           <t>2028E</t>
         </is>
@@ -1473,9 +1585,24 @@
           <t>Kinh doanh điện</t>
         </is>
       </c>
-      <c r="B2" s="22" t="inlineStr"/>
-      <c r="C2" s="22" t="inlineStr"/>
-      <c r="D2" s="22" t="inlineStr"/>
+      <c r="B2" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C2" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D2" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E2" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F2" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G2" s="23" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1483,9 +1610,24 @@
           <t>Cho thuê đất &amp; hạ tầng KCN</t>
         </is>
       </c>
-      <c r="B3" s="22" t="inlineStr"/>
-      <c r="C3" s="22" t="inlineStr"/>
-      <c r="D3" s="22" t="inlineStr"/>
+      <c r="B3" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C3" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D3" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E3" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F3" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G3" s="23" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1493,9 +1635,12 @@
           <t>Dịch vụ khu công nghiệp</t>
         </is>
       </c>
-      <c r="B4" s="22" t="inlineStr"/>
-      <c r="C4" s="22" t="inlineStr"/>
-      <c r="D4" s="22" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" s="24" t="inlineStr"/>
+      <c r="F4" s="24" t="inlineStr"/>
+      <c r="G4" s="24" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1503,9 +1648,24 @@
           <t>Thu phí đường bộ (BOT)</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr"/>
-      <c r="C5" s="22" t="inlineStr"/>
-      <c r="D5" s="22" t="inlineStr"/>
+      <c r="B5" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E5" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F5" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1513,9 +1673,24 @@
           <t>Hoạt động xây dựng</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr"/>
-      <c r="C6" s="22" t="inlineStr"/>
-      <c r="D6" s="22" t="inlineStr"/>
+      <c r="B6" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F6" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1523,9 +1698,24 @@
           <t>Kinh doanh BĐS</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr"/>
-      <c r="C7" s="22" t="inlineStr"/>
-      <c r="D7" s="22" t="inlineStr"/>
+      <c r="B7" s="18" t="n">
+        <v>0.2004</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E7" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1533,9 +1723,24 @@
           <t>Sản phẩm &amp; dịch vụ khác</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr"/>
-      <c r="C8" s="22" t="inlineStr"/>
-      <c r="D8" s="22" t="inlineStr"/>
+      <c r="B8" s="18" t="n">
+        <v>0.1429</v>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E8" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>0.2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1597,19 +1802,19 @@
           <t>Tiền &amp; tương đương</t>
         </is>
       </c>
-      <c r="B2" s="23" t="n">
+      <c r="B2" s="19" t="n">
         <v>495.13</v>
       </c>
-      <c r="C2" s="23" t="n">
+      <c r="C2" s="19" t="n">
         <v>1086.92</v>
       </c>
-      <c r="D2" s="23" t="n">
+      <c r="D2" s="19" t="n">
         <v>1333.59</v>
       </c>
-      <c r="E2" s="23" t="n">
+      <c r="E2" s="19" t="n">
         <v>2188.04</v>
       </c>
-      <c r="F2" s="23" t="n">
+      <c r="F2" s="19" t="n">
         <v>553.05</v>
       </c>
     </row>
@@ -1619,19 +1824,19 @@
           <t>Tổng tài sản</t>
         </is>
       </c>
-      <c r="B3" s="23" t="n">
+      <c r="B3" s="19" t="n">
         <v>16075.84</v>
       </c>
-      <c r="C3" s="23" t="n">
+      <c r="C3" s="19" t="n">
         <v>17013.41</v>
       </c>
-      <c r="D3" s="23" t="n">
+      <c r="D3" s="19" t="n">
         <v>17720.45</v>
       </c>
-      <c r="E3" s="23" t="n">
+      <c r="E3" s="19" t="n">
         <v>18800.16</v>
       </c>
-      <c r="F3" s="23" t="n">
+      <c r="F3" s="19" t="n">
         <v>23201.49</v>
       </c>
     </row>
@@ -1641,19 +1846,19 @@
           <t>Vay ngắn hạn</t>
         </is>
       </c>
-      <c r="B4" s="23" t="n">
+      <c r="B4" s="19" t="n">
         <v>1447.73</v>
       </c>
-      <c r="C4" s="23" t="n">
+      <c r="C4" s="19" t="n">
         <v>748.24</v>
       </c>
-      <c r="D4" s="23" t="n">
+      <c r="D4" s="19" t="n">
         <v>937.78</v>
       </c>
-      <c r="E4" s="23" t="n">
+      <c r="E4" s="19" t="n">
         <v>1143.72</v>
       </c>
-      <c r="F4" s="23" t="n">
+      <c r="F4" s="19" t="n">
         <v>2611.82</v>
       </c>
     </row>
@@ -1663,19 +1868,19 @@
           <t>Vay dài hạn</t>
         </is>
       </c>
-      <c r="B5" s="23" t="n">
+      <c r="B5" s="19" t="n">
         <v>2084.65</v>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="C5" s="19" t="n">
         <v>2719.53</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="19" t="n">
         <v>2584.73</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="19" t="n">
         <v>1992.31</v>
       </c>
-      <c r="F5" s="23" t="n">
+      <c r="F5" s="19" t="n">
         <v>3265.35</v>
       </c>
     </row>
@@ -1685,19 +1890,19 @@
           <t>Tổng nợ phải trả</t>
         </is>
       </c>
-      <c r="B6" s="23" t="n">
+      <c r="B6" s="19" t="n">
         <v>11047.8</v>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="19" t="n">
         <v>10885.49</v>
       </c>
-      <c r="D6" s="23" t="n">
+      <c r="D6" s="19" t="n">
         <v>11515.53</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="19" t="n">
         <v>11592.51</v>
       </c>
-      <c r="F6" s="23" t="n">
+      <c r="F6" s="19" t="n">
         <v>14938.46</v>
       </c>
     </row>
@@ -1707,19 +1912,19 @@
           <t>VCSH (bao gồm NCI)</t>
         </is>
       </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="19" t="n">
         <v>5028.04</v>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="19" t="n">
         <v>6127.92</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="19" t="n">
         <v>6204.91</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="19" t="n">
         <v>7207.65</v>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="19" t="n">
         <v>8263.030000000001</v>
       </c>
     </row>
@@ -1729,19 +1934,19 @@
           <t>Vốn góp (charter capital)</t>
         </is>
       </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="19" t="n">
         <v>3000</v>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="19" t="n">
         <v>3300</v>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="19" t="n">
         <v>3300</v>
       </c>
-      <c r="E8" s="23" t="n">
+      <c r="E8" s="19" t="n">
         <v>3300</v>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="19" t="n">
         <v>3794.99</v>
       </c>
     </row>
@@ -1751,24 +1956,24 @@
           <t>NCI (cổ đông thiểu số)</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n">
+      <c r="B9" s="19" t="n">
         <v>1128.37</v>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="19" t="n">
         <v>1181.86</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="19" t="n">
         <v>1232.22</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="19" t="n">
         <v>1591.82</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="19" t="n">
         <v>1803.66</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>VCSH cổ đông mẹ (= VCSH − NCI)</t>
         </is>
@@ -1795,19 +2000,19 @@
           <t>BVPS mẹ (VND/cp)</t>
         </is>
       </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="19" t="n">
         <v>12999</v>
       </c>
-      <c r="C12" s="23" t="n">
+      <c r="C12" s="19" t="n">
         <v>16487</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="19" t="n">
         <v>16576</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="19" t="n">
         <v>18719</v>
       </c>
-      <c r="F12" s="23" t="n">
+      <c r="F12" s="19" t="n">
         <v>21531</v>
       </c>
     </row>
@@ -1817,19 +2022,19 @@
           <t>EPS cơ bản (VND/cp)</t>
         </is>
       </c>
-      <c r="B13" s="23" t="n">
+      <c r="B13" s="19" t="n">
         <v>1514</v>
       </c>
-      <c r="C13" s="23" t="n">
+      <c r="C13" s="19" t="n">
         <v>5605</v>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D13" s="19" t="n">
         <v>4154</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E13" s="19" t="n">
         <v>5976</v>
       </c>
-      <c r="F13" s="23" t="n">
+      <c r="F13" s="19" t="n">
         <v>5090</v>
       </c>
     </row>
@@ -1892,12 +2097,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>─ COE &amp; CAPM ─</t>
         </is>
       </c>
-      <c r="B2" s="26" t="inlineStr"/>
+      <c r="B2" s="27" t="inlineStr"/>
       <c r="C2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
@@ -1923,12 +2128,12 @@
           <t>Beta</t>
         </is>
       </c>
-      <c r="B4" s="27" t="n">
-        <v>1.1511</v>
+      <c r="B4" s="28" t="n">
+        <v>1.1506</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Tự tính toán (1623 phiên)</t>
+          <t>Tự tính toán (1624 phiên)</t>
         </is>
       </c>
     </row>
@@ -1967,12 +2172,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>─ P/E ─</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr"/>
+      <c r="B7" s="27" t="inlineStr"/>
       <c r="C7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
@@ -1995,7 +2200,7 @@
           <t>P/E mục tiêu</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
+      <c r="B9" s="28" t="n">
         <v>8</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -2019,12 +2224,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>─ P/B ─</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr"/>
+      <c r="B11" s="27" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
@@ -2048,8 +2253,8 @@
           <t>P/B mục tiêu</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n">
-        <v>2.4</v>
+      <c r="B13" s="28" t="n">
+        <v>2.5</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -2064,7 +2269,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>54092</v>
+        <v>56346</v>
       </c>
       <c r="C14" s="3">
         <f> P/B × BVPS_fc1</f>
@@ -2072,12 +2277,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>─ Residual Income ─</t>
         </is>
       </c>
-      <c r="B15" s="26" t="inlineStr"/>
+      <c r="B15" s="27" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
@@ -2117,7 +2322,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>2979.6</v>
+        <v>2980.2</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
@@ -2132,7 +2337,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>3080.6</v>
+        <v>3081.3</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
@@ -2147,7 +2352,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>3171.3</v>
+        <v>3172</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
@@ -2162,7 +2367,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>37794.4</v>
+        <v>37820.1</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
@@ -2177,7 +2382,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>68557</v>
+        <v>68585</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
@@ -2186,12 +2391,12 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>─ KẾT QUẢ ─</t>
         </is>
       </c>
-      <c r="B23" s="26" t="inlineStr"/>
+      <c r="B23" s="27" t="inlineStr"/>
       <c r="C23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
@@ -2201,18 +2406,18 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>40000</v>
+        <v>40700</v>
       </c>
       <c r="C24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>Giá mục tiêu (40+40+20)</t>
         </is>
       </c>
       <c r="B25" s="10" t="n">
-        <v>53378</v>
+        <v>54285</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
@@ -2221,13 +2426,13 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="24" t="inlineStr">
+      <c r="A26" s="25" t="inlineStr">
         <is>
           <t>Upside / Downside</t>
         </is>
       </c>
-      <c r="B26" s="28" t="n">
-        <v>0.3345</v>
+      <c r="B26" s="29" t="n">
+        <v>0.3338</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
@@ -2246,16 +2451,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2271,25 +2477,30 @@
       </c>
       <c r="C1" s="12" t="inlineStr">
         <is>
+          <t>2025Q3</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
           <t>2026Q1</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>GV</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="G1" s="12" t="inlineStr">
         <is>
           <t>LNG</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="H1" s="12" t="inlineStr">
         <is>
           <t>Biên LNG</t>
         </is>
@@ -2301,23 +2512,26 @@
           <t>Kinh doanh điện</t>
         </is>
       </c>
-      <c r="B2" s="23" t="n">
+      <c r="B2" s="19" t="n">
         <v>815.7</v>
       </c>
-      <c r="C2" s="23" t="n">
+      <c r="C2" s="19" t="n">
+        <v>13.05</v>
+      </c>
+      <c r="D2" s="19" t="n">
         <v>883.8</v>
       </c>
-      <c r="D2" s="29" t="n">
-        <v>849.75</v>
-      </c>
-      <c r="E2" s="29" t="n">
-        <v>773.7</v>
-      </c>
-      <c r="F2" s="29" t="n">
-        <v>76.05</v>
+      <c r="E2" s="30" t="n">
+        <v>570.85</v>
+      </c>
+      <c r="F2" s="30" t="n">
+        <v>519.28</v>
       </c>
       <c r="G2" s="30" t="n">
-        <v>0.0895</v>
+        <v>51.57</v>
+      </c>
+      <c r="H2" s="31" t="n">
+        <v>0.09030000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -2326,23 +2540,26 @@
           <t>Cho thuê đất &amp; hạ tầng KCN</t>
         </is>
       </c>
-      <c r="B3" s="23" t="n">
+      <c r="B3" s="19" t="n">
         <v>467.5</v>
       </c>
-      <c r="C3" s="23" t="n">
+      <c r="C3" s="19" t="n">
+        <v>95.51000000000001</v>
+      </c>
+      <c r="D3" s="19" t="n">
         <v>268.9</v>
       </c>
-      <c r="D3" s="29" t="n">
-        <v>368.2</v>
-      </c>
-      <c r="E3" s="29" t="n">
-        <v>147.2</v>
-      </c>
-      <c r="F3" s="29" t="n">
-        <v>221</v>
+      <c r="E3" s="30" t="n">
+        <v>277.3</v>
+      </c>
+      <c r="F3" s="30" t="n">
+        <v>123.6</v>
       </c>
       <c r="G3" s="30" t="n">
-        <v>0.6002</v>
+        <v>153.7</v>
+      </c>
+      <c r="H3" s="31" t="n">
+        <v>0.5543</v>
       </c>
     </row>
     <row r="4">
@@ -2351,22 +2568,23 @@
           <t>Dịch vụ khu công nghiệp</t>
         </is>
       </c>
-      <c r="B4" s="23" t="n">
+      <c r="B4" s="19" t="n">
         <v>121.2</v>
       </c>
-      <c r="C4" s="23" t="n">
+      <c r="C4" s="19" t="inlineStr"/>
+      <c r="D4" s="19" t="n">
         <v>136.9</v>
       </c>
-      <c r="D4" s="29" t="n">
+      <c r="E4" s="30" t="n">
         <v>129.05</v>
       </c>
-      <c r="E4" s="29" t="n">
+      <c r="F4" s="30" t="n">
         <v>67.65000000000001</v>
       </c>
-      <c r="F4" s="29" t="n">
+      <c r="G4" s="30" t="n">
         <v>61.4</v>
       </c>
-      <c r="G4" s="30" t="n">
+      <c r="H4" s="31" t="n">
         <v>0.4758</v>
       </c>
     </row>
@@ -2376,23 +2594,26 @@
           <t>Thu phí đường bộ (BOT)</t>
         </is>
       </c>
-      <c r="B5" s="23" t="n">
+      <c r="B5" s="19" t="n">
         <v>112.7</v>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="C5" s="19" t="n">
+        <v>19.18</v>
+      </c>
+      <c r="D5" s="19" t="n">
         <v>120.3</v>
       </c>
-      <c r="D5" s="29" t="n">
-        <v>116.5</v>
-      </c>
-      <c r="E5" s="29" t="n">
-        <v>67.59999999999999</v>
-      </c>
-      <c r="F5" s="29" t="n">
-        <v>48.9</v>
+      <c r="E5" s="30" t="n">
+        <v>84.06</v>
+      </c>
+      <c r="F5" s="30" t="n">
+        <v>50.18</v>
       </c>
       <c r="G5" s="30" t="n">
-        <v>0.4197</v>
+        <v>33.88</v>
+      </c>
+      <c r="H5" s="31" t="n">
+        <v>0.403</v>
       </c>
     </row>
     <row r="6">
@@ -2401,23 +2622,26 @@
           <t>Hoạt động xây dựng</t>
         </is>
       </c>
-      <c r="B6" s="23" t="n">
+      <c r="B6" s="19" t="n">
         <v>37.8</v>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="19" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="D6" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="D6" s="29" t="n">
-        <v>34.4</v>
-      </c>
-      <c r="E6" s="29" t="n">
-        <v>46.25</v>
-      </c>
-      <c r="F6" s="29" t="n">
-        <v>-11.85</v>
+      <c r="E6" s="30" t="n">
+        <v>23.17</v>
+      </c>
+      <c r="F6" s="30" t="n">
+        <v>31.03</v>
       </c>
       <c r="G6" s="30" t="n">
-        <v>-0.3445</v>
+        <v>-7.85</v>
+      </c>
+      <c r="H6" s="31" t="n">
+        <v>-0.3388</v>
       </c>
     </row>
     <row r="7">
@@ -2426,23 +2650,26 @@
           <t>Kinh doanh BĐS</t>
         </is>
       </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="19" t="n">
         <v>182.2</v>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="19" t="n">
+        <v>72.33</v>
+      </c>
+      <c r="D7" s="19" t="n">
         <v>17.7</v>
       </c>
-      <c r="D7" s="29" t="n">
-        <v>99.95</v>
-      </c>
-      <c r="E7" s="29" t="n">
-        <v>30.3</v>
-      </c>
-      <c r="F7" s="29" t="n">
-        <v>69.65000000000001</v>
+      <c r="E7" s="30" t="n">
+        <v>90.73999999999999</v>
+      </c>
+      <c r="F7" s="30" t="n">
+        <v>39.49</v>
       </c>
       <c r="G7" s="30" t="n">
-        <v>0.6968</v>
+        <v>51.26</v>
+      </c>
+      <c r="H7" s="31" t="n">
+        <v>0.5649</v>
       </c>
     </row>
     <row r="8">
@@ -2451,23 +2678,26 @@
           <t>Sản phẩm &amp; dịch vụ khác</t>
         </is>
       </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="19" t="n">
         <v>56.5</v>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="19" t="n">
+        <v>2619.9</v>
+      </c>
+      <c r="D8" s="19" t="n">
         <v>27.1</v>
       </c>
-      <c r="D8" s="29" t="n">
-        <v>41.8</v>
-      </c>
-      <c r="E8" s="29" t="n">
-        <v>36.75</v>
-      </c>
-      <c r="F8" s="29" t="n">
-        <v>5.05</v>
+      <c r="E8" s="30" t="n">
+        <v>901.17</v>
+      </c>
+      <c r="F8" s="30" t="n">
+        <v>723.14</v>
       </c>
       <c r="G8" s="30" t="n">
-        <v>0.1208</v>
+        <v>178.03</v>
+      </c>
+      <c r="H8" s="31" t="n">
+        <v>0.1976</v>
       </c>
     </row>
   </sheetData>

</xml_diff>